<commit_message>
Swap four AliExpress parts to Choice listings
Single-seller listings each charged $4-6 shipping; Choice items ship
together. Radar, RTC, USB-C board and light sensor updated in the
spreadsheet and PARTS.md.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Sunrise_Clock_Parts.xlsx
+++ b/Sunrise_Clock_Parts.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\asher\AppData\Local\Temp\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{35999A17-B4D0-4AE3-94BA-9A056BA8036E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CAA4B1CA-8D93-45C8-B9B2-20E03FA47C8B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1520" yWindow="1520" windowWidth="19200" windowHeight="11170" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -60,12 +60,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="157" uniqueCount="129">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="160" uniqueCount="134">
   <si>
     <t>Sunrise Clock: parts, Amazon vs AliExpress</t>
   </si>
   <si>
-    <t>One clock, every function. Prices checked 2026-10-20 on amazon.com and aliexpress.us (AliExpress: regular price, not the one-time new-shopper deal). Prices change. ESP32 and PLA not included (you have them).</t>
+    <t>One clock, every function. Prices checked 2026-10-20 on amazon.com and aliexpress.us (AliExpress: regular price, not the one-time new-shopper deal). Prices change. ESP32 and PLA not included (you have them). AliExpress 'Choice' items ship together, free once they total about $10; other AliExpress sellers each charge shipping.</t>
   </si>
   <si>
     <t>Part</t>
@@ -236,10 +236,13 @@
     <t>4.4★</t>
   </si>
   <si>
-    <t>4.9★, 900+ sold</t>
-  </si>
-  <si>
-    <t>DS3231SN</t>
+    <t>1 pc, Choice</t>
+  </si>
+  <si>
+    <t>4.8★, 4,000+ sold, Choice</t>
+  </si>
+  <si>
+    <t>DS3231SN, blue board with coin-cell holder</t>
   </si>
   <si>
     <t>DS3231M chips are less accurate but still work. Remove the charging resistor for a CR2032.</t>
@@ -287,13 +290,16 @@
     <t>no reviews yet</t>
   </si>
   <si>
-    <t>dual 5.1K board</t>
-  </si>
-  <si>
-    <t>4.8★, 2,000+ sold</t>
-  </si>
-  <si>
-    <t>AliExpress listing is the proven one here</t>
+    <t>Type-C board, CC1/CC2 5.1K, Choice</t>
+  </si>
+  <si>
+    <t>5★, 347 sold, Choice</t>
+  </si>
+  <si>
+    <t>with 5.1K resistors</t>
+  </si>
+  <si>
+    <t>AliExpress listing has the better track record here</t>
   </si>
   <si>
     <t>HLK-LD2410C sleep radar</t>
@@ -305,7 +311,10 @@
     <t>4.6★, 9 reviews</t>
   </si>
   <si>
-    <t>571 sold</t>
+    <t>4.8★, 5,000+ sold, Choice</t>
+  </si>
+  <si>
+    <t>LD2410C (not B or 2420)</t>
   </si>
   <si>
     <t>Same Hi-Link module. Pocket is 22 × 16 mm: measure yours.</t>
@@ -392,7 +401,13 @@
     <t>HiLetgo 3 pcs</t>
   </si>
   <si>
-    <t>516 sold</t>
+    <t>GY-302, Choice</t>
+  </si>
+  <si>
+    <t>5★, 414 sold, Choice</t>
+  </si>
+  <si>
+    <t>GY-302</t>
   </si>
   <si>
     <t>Only needed for auto-dim</t>
@@ -440,7 +455,7 @@
     <t>Yellow cells (My pick): choose Amazon, AliExpress or None from the dropdown. My price and its total update.</t>
   </si>
   <si>
-    <t>Blue numbers are prices typed in from the listings on 2026-10-20; black numbers are formulas.</t>
+    <t>Blue numbers are prices typed in from the listings on 2026-10-20 (Choice swaps 2026-10-21); black numbers are formulas.</t>
   </si>
   <si>
     <t>Click a listing name to open it. On AliExpress, choose the option in the 'AliExpress option to pick' column.</t>
@@ -1261,7 +1276,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="11" spans="1:13" ht="28" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:13" ht="42" x14ac:dyDescent="0.35">
       <c r="A11" s="3" t="s">
         <v>55</v>
       </c>
@@ -1278,35 +1293,35 @@
         <v>57</v>
       </c>
       <c r="F11" s="4" t="s">
-        <v>44</v>
+        <v>58</v>
       </c>
       <c r="G11" s="5">
-        <v>2.83</v>
+        <v>3.14</v>
       </c>
       <c r="H11" s="3" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="I11" s="3" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="J11" s="6">
         <f t="shared" si="0"/>
-        <v>5.16</v>
+        <v>4.8499999999999996</v>
       </c>
       <c r="K11" s="7" t="s">
         <v>21</v>
       </c>
       <c r="L11" s="6">
         <f t="shared" si="1"/>
-        <v>2.83</v>
+        <v>3.14</v>
       </c>
       <c r="M11" s="3" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
     </row>
     <row r="12" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A12" s="3" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="B12" s="3">
         <v>1</v>
@@ -1321,13 +1336,13 @@
         <v>43</v>
       </c>
       <c r="F12" s="4" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="G12" s="5">
         <v>1.48</v>
       </c>
       <c r="H12" s="3" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="I12" s="3"/>
       <c r="J12" s="6">
@@ -1342,36 +1357,36 @@
         <v>1.48</v>
       </c>
       <c r="M12" s="3" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
     </row>
     <row r="13" spans="1:13" ht="28" x14ac:dyDescent="0.35">
       <c r="A13" s="3" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="B13" s="3">
         <v>2</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="D13" s="5">
         <v>7.99</v>
       </c>
       <c r="E13" s="3" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="F13" s="4" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="G13" s="5">
         <v>4.4000000000000004</v>
       </c>
       <c r="H13" s="3" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="I13" s="3" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="J13" s="6">
         <f t="shared" si="0"/>
@@ -1385,100 +1400,104 @@
         <v>7.99</v>
       </c>
       <c r="M13" s="3" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="14" spans="1:13" x14ac:dyDescent="0.35">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="14" spans="1:13" ht="28" x14ac:dyDescent="0.35">
       <c r="A14" s="3" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="B14" s="3">
         <v>1</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="D14" s="5">
         <v>8.9</v>
       </c>
       <c r="E14" s="3" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="F14" s="4" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="G14" s="5">
-        <v>0.41</v>
+        <v>2.86</v>
       </c>
       <c r="H14" s="3" t="s">
-        <v>76</v>
-      </c>
-      <c r="I14" s="3"/>
+        <v>77</v>
+      </c>
+      <c r="I14" s="3" t="s">
+        <v>78</v>
+      </c>
       <c r="J14" s="6">
         <f t="shared" si="0"/>
-        <v>8.49</v>
+        <v>6.0400000000000009</v>
       </c>
       <c r="K14" s="7" t="s">
         <v>21</v>
       </c>
       <c r="L14" s="6">
         <f t="shared" si="1"/>
-        <v>0.41</v>
+        <v>2.86</v>
       </c>
       <c r="M14" s="3" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="15" spans="1:13" x14ac:dyDescent="0.35">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="15" spans="1:13" ht="28" x14ac:dyDescent="0.35">
       <c r="A15" s="3" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="B15" s="3">
         <v>1</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="D15" s="5">
         <v>13.99</v>
       </c>
       <c r="E15" s="3" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="F15" s="4" t="s">
-        <v>44</v>
+        <v>58</v>
       </c>
       <c r="G15" s="5">
-        <v>4.1900000000000004</v>
+        <v>5.91</v>
       </c>
       <c r="H15" s="3" t="s">
-        <v>81</v>
-      </c>
-      <c r="I15" s="3"/>
+        <v>83</v>
+      </c>
+      <c r="I15" s="3" t="s">
+        <v>84</v>
+      </c>
       <c r="J15" s="6">
         <f t="shared" si="0"/>
-        <v>9.8000000000000007</v>
+        <v>8.08</v>
       </c>
       <c r="K15" s="7" t="s">
         <v>21</v>
       </c>
       <c r="L15" s="6">
         <f t="shared" si="1"/>
-        <v>4.1900000000000004</v>
+        <v>5.91</v>
       </c>
       <c r="M15" s="3" t="s">
-        <v>82</v>
+        <v>85</v>
       </c>
     </row>
     <row r="16" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A16" s="3" t="s">
-        <v>83</v>
+        <v>86</v>
       </c>
       <c r="B16" s="3">
         <v>1</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>84</v>
+        <v>87</v>
       </c>
       <c r="D16" s="5">
         <v>3.99</v>
@@ -1487,14 +1506,14 @@
         <v>38</v>
       </c>
       <c r="F16" s="4" t="s">
-        <v>85</v>
+        <v>88</v>
       </c>
       <c r="G16" s="5">
         <v>3.32</v>
       </c>
       <c r="H16" s="3"/>
       <c r="I16" s="3" t="s">
-        <v>86</v>
+        <v>89</v>
       </c>
       <c r="J16" s="6">
         <f t="shared" si="0"/>
@@ -1508,18 +1527,18 @@
         <v>3.32</v>
       </c>
       <c r="M16" s="3" t="s">
-        <v>87</v>
+        <v>90</v>
       </c>
     </row>
     <row r="17" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A17" s="3" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="B17" s="3">
         <v>1</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
       <c r="D17" s="5">
         <v>13.99</v>
@@ -1534,10 +1553,10 @@
         <v>4.1500000000000004</v>
       </c>
       <c r="H17" s="3" t="s">
-        <v>90</v>
+        <v>93</v>
       </c>
       <c r="I17" s="3" t="s">
-        <v>91</v>
+        <v>94</v>
       </c>
       <c r="J17" s="6">
         <f t="shared" si="0"/>
@@ -1551,18 +1570,18 @@
         <v>4.1500000000000004</v>
       </c>
       <c r="M17" s="3" t="s">
-        <v>92</v>
+        <v>95</v>
       </c>
     </row>
     <row r="18" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A18" s="3" t="s">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="B18" s="3">
         <v>1</v>
       </c>
       <c r="C18" s="4" t="s">
-        <v>94</v>
+        <v>97</v>
       </c>
       <c r="D18" s="5">
         <v>5.99</v>
@@ -1571,16 +1590,16 @@
         <v>25</v>
       </c>
       <c r="F18" s="4" t="s">
-        <v>95</v>
+        <v>98</v>
       </c>
       <c r="G18" s="5">
         <v>2.71</v>
       </c>
       <c r="H18" s="3" t="s">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="I18" s="3" t="s">
-        <v>97</v>
+        <v>100</v>
       </c>
       <c r="J18" s="6">
         <f t="shared" si="0"/>
@@ -1594,36 +1613,36 @@
         <v>2.71</v>
       </c>
       <c r="M18" s="3" t="s">
-        <v>98</v>
+        <v>101</v>
       </c>
     </row>
     <row r="19" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A19" s="3" t="s">
-        <v>99</v>
+        <v>102</v>
       </c>
       <c r="B19" s="3">
         <v>1</v>
       </c>
       <c r="C19" s="4" t="s">
-        <v>100</v>
+        <v>103</v>
       </c>
       <c r="D19" s="5">
         <v>8.99</v>
       </c>
       <c r="E19" s="3" t="s">
-        <v>101</v>
+        <v>104</v>
       </c>
       <c r="F19" s="4" t="s">
-        <v>102</v>
+        <v>105</v>
       </c>
       <c r="G19" s="5">
         <v>5.65</v>
       </c>
       <c r="H19" s="3" t="s">
-        <v>103</v>
+        <v>106</v>
       </c>
       <c r="I19" s="3" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="J19" s="6">
         <f t="shared" si="0"/>
@@ -1637,12 +1656,12 @@
         <v>5.65</v>
       </c>
       <c r="M19" s="3" t="s">
-        <v>87</v>
+        <v>90</v>
       </c>
     </row>
     <row r="20" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A20" s="8" t="s">
-        <v>105</v>
+        <v>108</v>
       </c>
       <c r="B20" s="9"/>
       <c r="C20" s="9"/>
@@ -1654,37 +1673,37 @@
       <c r="F20" s="9"/>
       <c r="G20" s="10">
         <f>SUM(G5:G19)</f>
-        <v>50.410000000000004</v>
+        <v>54.89</v>
       </c>
       <c r="H20" s="9"/>
       <c r="I20" s="9"/>
       <c r="J20" s="10">
         <f>SUM(J5:J19)</f>
-        <v>79.140000000000015</v>
+        <v>74.660000000000011</v>
       </c>
       <c r="K20" s="9"/>
       <c r="L20" s="10">
         <f>SUM(L5:L19)</f>
-        <v>58.149999999999991</v>
+        <v>62.629999999999995</v>
       </c>
       <c r="M20" s="11" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
     </row>
     <row r="22" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A22" s="12" t="s">
-        <v>107</v>
+        <v>110</v>
       </c>
     </row>
     <row r="23" spans="1:13" ht="28" x14ac:dyDescent="0.35">
       <c r="A23" s="3" t="s">
-        <v>108</v>
+        <v>111</v>
       </c>
       <c r="B23" s="3">
         <v>1</v>
       </c>
       <c r="C23" s="4" t="s">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="D23" s="5">
         <v>7.49</v>
@@ -1693,33 +1712,35 @@
         <v>43</v>
       </c>
       <c r="F23" s="4" t="s">
-        <v>44</v>
+        <v>113</v>
       </c>
       <c r="G23" s="5">
-        <v>4.05</v>
+        <v>2.19</v>
       </c>
       <c r="H23" s="3" t="s">
-        <v>110</v>
-      </c>
-      <c r="I23" s="3"/>
+        <v>114</v>
+      </c>
+      <c r="I23" s="3" t="s">
+        <v>115</v>
+      </c>
       <c r="J23" s="6">
         <f>D23-G23</f>
-        <v>3.4400000000000004</v>
+        <v>5.3000000000000007</v>
       </c>
       <c r="K23" s="7" t="s">
         <v>21</v>
       </c>
       <c r="L23" s="6">
         <f>IF(K23="Amazon",D23,IF(K23="AliExpress",G23,0))</f>
-        <v>4.05</v>
+        <v>2.19</v>
       </c>
       <c r="M23" s="3" t="s">
-        <v>111</v>
+        <v>116</v>
       </c>
     </row>
     <row r="24" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A24" s="8" t="s">
-        <v>112</v>
+        <v>117</v>
       </c>
       <c r="B24" s="9"/>
       <c r="C24" s="9"/>
@@ -1731,29 +1752,29 @@
       <c r="F24" s="9"/>
       <c r="G24" s="10">
         <f>G20+SUM(G23:G23)</f>
-        <v>54.46</v>
+        <v>57.08</v>
       </c>
       <c r="H24" s="9"/>
       <c r="I24" s="9"/>
       <c r="J24" s="10">
         <f>J20+SUM(J23:J23)</f>
-        <v>82.580000000000013</v>
+        <v>79.960000000000008</v>
       </c>
       <c r="K24" s="9"/>
       <c r="L24" s="10">
         <f>L20+SUM(L23:L23)</f>
-        <v>62.199999999999989</v>
+        <v>64.819999999999993</v>
       </c>
       <c r="M24" s="9"/>
     </row>
     <row r="26" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A26" s="12" t="s">
-        <v>113</v>
+        <v>118</v>
       </c>
     </row>
     <row r="27" spans="1:13" ht="28" x14ac:dyDescent="0.35">
       <c r="A27" s="4" t="s">
-        <v>114</v>
+        <v>119</v>
       </c>
       <c r="B27" s="13"/>
       <c r="C27" s="13"/>
@@ -1769,12 +1790,12 @@
       <c r="K27" s="13"/>
       <c r="L27" s="13"/>
       <c r="M27" s="3" t="s">
-        <v>115</v>
+        <v>120</v>
       </c>
     </row>
     <row r="28" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A28" s="4" t="s">
-        <v>116</v>
+        <v>121</v>
       </c>
       <c r="B28" s="13"/>
       <c r="C28" s="13"/>
@@ -1790,12 +1811,12 @@
       <c r="K28" s="13"/>
       <c r="L28" s="13"/>
       <c r="M28" s="3" t="s">
-        <v>117</v>
+        <v>122</v>
       </c>
     </row>
     <row r="29" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A29" s="4" t="s">
-        <v>118</v>
+        <v>123</v>
       </c>
       <c r="B29" s="13"/>
       <c r="C29" s="13"/>
@@ -1811,12 +1832,12 @@
       <c r="K29" s="13"/>
       <c r="L29" s="13"/>
       <c r="M29" s="3" t="s">
-        <v>119</v>
+        <v>124</v>
       </c>
     </row>
     <row r="30" spans="1:13" ht="28" x14ac:dyDescent="0.35">
       <c r="A30" s="4" t="s">
-        <v>120</v>
+        <v>125</v>
       </c>
       <c r="B30" s="13"/>
       <c r="C30" s="13"/>
@@ -1832,12 +1853,12 @@
       <c r="K30" s="13"/>
       <c r="L30" s="13"/>
       <c r="M30" s="3" t="s">
-        <v>121</v>
+        <v>126</v>
       </c>
     </row>
     <row r="31" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A31" s="4" t="s">
-        <v>122</v>
+        <v>127</v>
       </c>
       <c r="B31" s="13"/>
       <c r="C31" s="13"/>
@@ -1853,32 +1874,32 @@
       <c r="K31" s="13"/>
       <c r="L31" s="13"/>
       <c r="M31" s="3" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
     </row>
     <row r="33" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A33" s="14" t="s">
-        <v>124</v>
+        <v>129</v>
       </c>
     </row>
     <row r="34" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A34" s="15" t="s">
-        <v>125</v>
+        <v>130</v>
       </c>
     </row>
     <row r="35" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A35" s="15" t="s">
-        <v>126</v>
+        <v>131</v>
       </c>
     </row>
     <row r="36" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A36" s="15" t="s">
-        <v>127</v>
+        <v>132</v>
       </c>
     </row>
     <row r="37" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A37" s="15" t="s">
-        <v>128</v>
+        <v>133</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Workbook: fix circular totals and stale Parts-tab cells
Parts row 16 summed rows 5-30, which included itself, so its totals
came out blank. It now sums the part rows plus the inserts and
screws. The Parts tab also gets the $4.75 strip price, the Flat Head
button link, and the M3 OD 4.5 x 5 mm insert at $3.40, matching the
Buying tab.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Sunrise_Clock_Parts.xlsx
+++ b/Sunrise_Clock_Parts.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\asher\AppData\Local\Temp\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D08BD59C-0B72-4114-B13F-53635DDF17EC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{12996AC7-117F-4DBA-A487-D5AE3A9028EE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="6400" yWindow="2250" windowWidth="19200" windowHeight="11170" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -391,6 +391,9 @@
     <t>Same module, with the pull-ups GPIO34/35 need</t>
   </si>
   <si>
+    <t>Gebildet 5 pcs, Flat Head (SS-Momentary-5pcs)</t>
+  </si>
+  <si>
     <t>4.6★, 981 reviews</t>
   </si>
   <si>
@@ -502,10 +505,7 @@
     <t>54,000+ sold</t>
   </si>
   <si>
-    <t>M3 x 5.7 x 4.6</t>
-  </si>
-  <si>
-    <t>Amazon's size is confirmed; on Ali pick M3 × 5.7 × 4.6 if offered</t>
+    <t>Holes are Ø4.0 × 5 mm: a 5 mm insert sits flush. OD 5 mm or wider can split the posts.</t>
   </si>
   <si>
     <t>4.8★, 1,000+ sold</t>
@@ -1094,7 +1094,7 @@
       </c>
       <c r="E1" s="17">
         <f>SUM(G5:G7,G9:G10,G12:G15,D8,D11,G19)</f>
-        <v>51.870000000000005</v>
+        <v>52.03</v>
       </c>
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.35">
@@ -1175,7 +1175,7 @@
         <v>10</v>
       </c>
       <c r="G5" s="5">
-        <v>4.59</v>
+        <v>4.75</v>
       </c>
       <c r="H5" s="3" t="s">
         <v>87</v>
@@ -1185,14 +1185,14 @@
       </c>
       <c r="J5" s="6">
         <f t="shared" ref="J5:J15" si="0">D5-G5</f>
-        <v>7.4</v>
+        <v>7.24</v>
       </c>
       <c r="K5" s="7" t="s">
         <v>11</v>
       </c>
       <c r="L5" s="6">
         <f t="shared" ref="L5:L15" si="1">IF(K5="Amazon",D5,IF(K5="AliExpress",G5,0))</f>
-        <v>4.59</v>
+        <v>4.75</v>
       </c>
       <c r="M5" s="3" t="s">
         <v>89</v>
@@ -1417,25 +1417,25 @@
         <v>2</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>29</v>
+        <v>109</v>
       </c>
       <c r="D11" s="5">
         <v>7.99</v>
       </c>
       <c r="E11" s="3" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="F11" s="4" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="G11" s="5">
         <v>4.4000000000000004</v>
       </c>
       <c r="H11" s="3" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="I11" s="3" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="J11" s="6">
         <f t="shared" si="0"/>
@@ -1449,7 +1449,7 @@
         <v>7.99</v>
       </c>
       <c r="M11" s="3" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
     </row>
     <row r="12" spans="1:13" ht="28" customHeight="1" x14ac:dyDescent="0.35">
@@ -1460,13 +1460,13 @@
         <v>1</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="D12" s="5">
         <v>8.9</v>
       </c>
       <c r="E12" s="3" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="F12" s="4" t="s">
         <v>32</v>
@@ -1475,10 +1475,10 @@
         <v>2.86</v>
       </c>
       <c r="H12" s="3" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="I12" s="3" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="J12" s="6">
         <f t="shared" si="0"/>
@@ -1492,7 +1492,7 @@
         <v>2.86</v>
       </c>
       <c r="M12" s="3" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
     </row>
     <row r="13" spans="1:13" ht="28" customHeight="1" x14ac:dyDescent="0.35">
@@ -1503,13 +1503,13 @@
         <v>1</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="D13" s="5">
         <v>13.99</v>
       </c>
       <c r="E13" s="3" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="F13" s="4" t="s">
         <v>24</v>
@@ -1518,10 +1518,10 @@
         <v>5.91</v>
       </c>
       <c r="H13" s="3" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="I13" s="3" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="J13" s="6">
         <f t="shared" si="0"/>
@@ -1535,7 +1535,7 @@
         <v>5.91</v>
       </c>
       <c r="M13" s="3" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
     </row>
     <row r="14" spans="1:13" x14ac:dyDescent="0.35">
@@ -1546,13 +1546,13 @@
         <v>1</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="D14" s="5">
         <v>3.99</v>
       </c>
       <c r="E14" s="3" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="F14" s="4" t="s">
         <v>37</v>
@@ -1562,7 +1562,7 @@
       </c>
       <c r="H14" s="3"/>
       <c r="I14" s="3" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="J14" s="6">
         <f t="shared" si="0"/>
@@ -1576,7 +1576,7 @@
         <v>3.32</v>
       </c>
       <c r="M14" s="3" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
     </row>
     <row r="15" spans="1:13" x14ac:dyDescent="0.35">
@@ -1587,7 +1587,7 @@
         <v>1</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="D15" s="5">
         <v>13.99</v>
@@ -1602,10 +1602,10 @@
         <v>4.1500000000000004</v>
       </c>
       <c r="H15" s="3" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="I15" s="3" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="J15" s="6">
         <f t="shared" si="0"/>
@@ -1619,7 +1619,7 @@
         <v>4.1500000000000004</v>
       </c>
       <c r="M15" s="3" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
     </row>
     <row r="16" spans="1:13" x14ac:dyDescent="0.35">
@@ -1628,34 +1628,34 @@
       </c>
       <c r="B16" s="9"/>
       <c r="C16" s="9"/>
-      <c r="D16" s="10" t="str">
-        <f ca="1">SUM(D5:D30)</f>
-        <v/>
+      <c r="D16" s="10">
+        <f>SUM(D5:D15,D29:D30)</f>
+        <v>119.56999999999998</v>
       </c>
       <c r="E16" s="9"/>
       <c r="F16" s="9"/>
-      <c r="G16" s="10" t="str">
-        <f ca="1">SUM(G5:G30)</f>
-        <v/>
+      <c r="G16" s="10">
+        <f>SUM(G5:G15,G29:G30)</f>
+        <v>51.149999999999991</v>
       </c>
       <c r="H16" s="9"/>
       <c r="I16" s="9"/>
-      <c r="J16" s="10" t="str">
-        <f ca="1">SUM(J5:J30)</f>
-        <v/>
+      <c r="J16" s="10">
+        <f>SUM(J5:J15,J29:J30)</f>
+        <v>68.42</v>
       </c>
       <c r="K16" s="9"/>
-      <c r="L16" s="10" t="str">
-        <f ca="1">SUM(L5:L30)</f>
-        <v/>
+      <c r="L16" s="10">
+        <f>SUM(L5:L15,L29:L30)</f>
+        <v>58.89</v>
       </c>
       <c r="M16" s="11" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
     </row>
     <row r="18" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A18" s="12" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
     </row>
     <row r="19" spans="1:13" ht="28" customHeight="1" x14ac:dyDescent="0.35">
@@ -1666,7 +1666,7 @@
         <v>1</v>
       </c>
       <c r="C19" s="4" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="D19" s="5">
         <v>7.49</v>
@@ -1681,10 +1681,10 @@
         <v>2.19</v>
       </c>
       <c r="H19" s="3" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="I19" s="3" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="J19" s="6">
         <f>D19-G19</f>
@@ -1698,7 +1698,7 @@
         <v>2.19</v>
       </c>
       <c r="M19" s="3" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
     </row>
     <row r="20" spans="1:13" x14ac:dyDescent="0.35">
@@ -1707,26 +1707,26 @@
       </c>
       <c r="B20" s="9"/>
       <c r="C20" s="9"/>
-      <c r="D20" s="10" t="str">
-        <f ca="1">D16+SUM(D19:D19)</f>
-        <v/>
+      <c r="D20" s="10">
+        <f>D16+SUM(D19:D19)</f>
+        <v>127.05999999999997</v>
       </c>
       <c r="E20" s="9"/>
       <c r="F20" s="9"/>
-      <c r="G20" s="10" t="str">
-        <f ca="1">G16+SUM(G19:G19)</f>
-        <v/>
+      <c r="G20" s="10">
+        <f>G16+SUM(G19:G19)</f>
+        <v>53.339999999999989</v>
       </c>
       <c r="H20" s="9"/>
       <c r="I20" s="9"/>
-      <c r="J20" s="10" t="str">
-        <f ca="1">J16+SUM(J19:J19)</f>
-        <v/>
+      <c r="J20" s="10">
+        <f>J16+SUM(J19:J19)</f>
+        <v>73.72</v>
       </c>
       <c r="K20" s="9"/>
-      <c r="L20" s="10" t="str">
-        <f ca="1">L16+SUM(L19:L19)</f>
-        <v/>
+      <c r="L20" s="10">
+        <f>L16+SUM(L19:L19)</f>
+        <v>61.08</v>
       </c>
       <c r="M20" s="9"/>
     </row>
@@ -1737,7 +1737,7 @@
     </row>
     <row r="23" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A23" s="16" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
     </row>
     <row r="24" spans="1:13" ht="28" customHeight="1" x14ac:dyDescent="0.35">
@@ -1758,7 +1758,7 @@
       <c r="K24" s="13"/>
       <c r="L24" s="13"/>
       <c r="M24" s="3" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
     </row>
     <row r="25" spans="1:13" x14ac:dyDescent="0.35">
@@ -1779,7 +1779,7 @@
       <c r="K25" s="13"/>
       <c r="L25" s="13"/>
       <c r="M25" s="3" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
     </row>
     <row r="26" spans="1:13" x14ac:dyDescent="0.35">
@@ -1802,7 +1802,7 @@
       <c r="K26" s="13"/>
       <c r="L26" s="13"/>
       <c r="M26" s="3" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
     </row>
     <row r="27" spans="1:13" ht="28" customHeight="1" x14ac:dyDescent="0.35">
@@ -1825,7 +1825,7 @@
       <c r="K27" s="13"/>
       <c r="L27" s="13"/>
       <c r="M27" s="3" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
     </row>
     <row r="28" spans="1:13" x14ac:dyDescent="0.35">
@@ -1848,10 +1848,10 @@
       <c r="K28" s="13"/>
       <c r="L28" s="13"/>
       <c r="M28" s="3" t="s">
-        <v>143</v>
-      </c>
-    </row>
-    <row r="29" spans="1:13" x14ac:dyDescent="0.35">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="29" spans="1:13" ht="42" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A29" s="3" t="s">
         <v>41</v>
       </c>
@@ -1859,7 +1859,7 @@
         <v>1</v>
       </c>
       <c r="C29" s="4" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="D29" s="5">
         <v>5.99</v>
@@ -1871,24 +1871,24 @@
         <v>42</v>
       </c>
       <c r="G29" s="5">
-        <v>2.71</v>
+        <v>3.4</v>
       </c>
       <c r="H29" s="3" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="I29" s="3" t="s">
-        <v>146</v>
+        <v>43</v>
       </c>
       <c r="J29" s="6">
         <f>D29-G29</f>
-        <v>3.2800000000000002</v>
+        <v>2.5900000000000003</v>
       </c>
       <c r="K29" s="7" t="s">
         <v>11</v>
       </c>
       <c r="L29" s="6">
         <f>IF(K29="Amazon",D29,IF(K29="AliExpress",G29,0))</f>
-        <v>2.71</v>
+        <v>3.4</v>
       </c>
       <c r="M29" s="3" t="s">
         <v>147</v>
@@ -1934,7 +1934,7 @@
         <v>5.65</v>
       </c>
       <c r="M30" s="3" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
     </row>
     <row r="31" spans="1:13" x14ac:dyDescent="0.35">

</xml_diff>